<commit_message>
Added config option to change the inventory target logic. Need to update the shortages and excesses logic accordingly too. The transfers are fine.
</commit_message>
<xml_diff>
--- a/outputs/inventory_summary.xlsx
+++ b/outputs/inventory_summary.xlsx
@@ -14151,10 +14151,10 @@
         <v>12.59328358208955</v>
       </c>
       <c r="H476">
-        <v>173.82</v>
+        <v>174.89</v>
       </c>
       <c r="I476">
-        <v>20.26819029850746</v>
+        <v>20.39295708955224</v>
       </c>
     </row>
     <row r="477" spans="1:9">
@@ -14180,10 +14180,10 @@
         <v>13.14501468326108</v>
       </c>
       <c r="H477">
-        <v>1739.21</v>
+        <v>1750</v>
       </c>
       <c r="I477">
-        <v>20.26767818020789</v>
+        <v>20.39341816995292</v>
       </c>
     </row>
     <row r="478" spans="1:9">
@@ -14238,10 +14238,10 @@
         <v>15.39179104477612</v>
       </c>
       <c r="H479">
-        <v>173.82</v>
+        <v>174.89</v>
       </c>
       <c r="I479">
-        <v>20.26819029850746</v>
+        <v>20.39295708955224</v>
       </c>
     </row>
     <row r="480" spans="1:9">
@@ -14296,10 +14296,10 @@
         <v>24.78347768154564</v>
       </c>
       <c r="H481">
-        <v>636.46</v>
+        <v>630.42</v>
       </c>
       <c r="I481">
-        <v>21.20119920053298</v>
+        <v>21</v>
       </c>
     </row>
     <row r="482" spans="1:9">
@@ -14325,10 +14325,10 @@
         <v>30.78358208955224</v>
       </c>
       <c r="H482">
-        <v>132</v>
+        <v>90.06</v>
       </c>
       <c r="I482">
-        <v>30.78358208955224</v>
+        <v>21.00279850746269</v>
       </c>
     </row>
     <row r="483" spans="1:9">
@@ -14354,7 +14354,7 @@
         <v>55.40011191941802</v>
       </c>
       <c r="H483">
-        <v>450.3200000000001</v>
+        <v>450.3199999999999</v>
       </c>
       <c r="I483">
         <v>20.99981346763663</v>
@@ -14412,10 +14412,10 @@
         <v>17.34023213536568</v>
       </c>
       <c r="H485">
-        <v>1739.21</v>
+        <v>1750</v>
       </c>
       <c r="I485">
-        <v>20.26767818020789</v>
+        <v>20.39341816995292</v>
       </c>
     </row>
     <row r="486" spans="1:9">
@@ -14441,10 +14441,10 @@
         <v>14.89696267483241</v>
       </c>
       <c r="H486">
-        <v>1959.16</v>
+        <v>1971.31</v>
       </c>
       <c r="I486">
-        <v>20.26773152362824</v>
+        <v>20.39342464619714</v>
       </c>
     </row>
     <row r="487" spans="1:9">
@@ -14528,10 +14528,10 @@
         <v>14.99516285069332</v>
       </c>
       <c r="H489">
-        <v>502.8</v>
+        <v>505.92</v>
       </c>
       <c r="I489">
-        <v>20.26765559496937</v>
+        <v>20.39342147694292</v>
       </c>
     </row>
     <row r="490" spans="1:9">
@@ -14557,10 +14557,10 @@
         <v>16.95294578414368</v>
       </c>
       <c r="H490">
-        <v>1448.98</v>
+        <v>1457.97</v>
       </c>
       <c r="I490">
-        <v>20.26772226263078</v>
+        <v>20.39347059810888</v>
       </c>
     </row>
     <row r="491" spans="1:9">
@@ -18199,10 +18199,7 @@
         <v>999999</v>
       </c>
       <c r="H616">
-        <v>648</v>
-      </c>
-      <c r="I616">
-        <v>999999</v>
+        <v>524.83</v>
       </c>
     </row>
     <row r="617" spans="1:9">
@@ -18228,10 +18225,7 @@
         <v>999999</v>
       </c>
       <c r="H617">
-        <v>192</v>
-      </c>
-      <c r="I617">
-        <v>999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="618" spans="1:9">
@@ -18257,10 +18251,10 @@
         <v>0</v>
       </c>
       <c r="H618">
-        <v>0</v>
+        <v>90.05</v>
       </c>
       <c r="I618">
-        <v>0</v>
+        <v>21.00046641791045</v>
       </c>
     </row>
     <row r="619" spans="1:9">
@@ -18286,10 +18280,10 @@
         <v>0</v>
       </c>
       <c r="H619">
-        <v>0</v>
+        <v>90.05</v>
       </c>
       <c r="I619">
-        <v>0</v>
+        <v>21.00046641791045</v>
       </c>
     </row>
     <row r="620" spans="1:9">
@@ -18315,10 +18309,10 @@
         <v>0</v>
       </c>
       <c r="H620">
-        <v>0</v>
+        <v>135.07</v>
       </c>
       <c r="I620">
-        <v>0</v>
+        <v>20.99968905472637</v>
       </c>
     </row>
     <row r="621" spans="1:9">
@@ -18346,9 +18340,6 @@
       <c r="H621">
         <v>492</v>
       </c>
-      <c r="I621">
-        <v>999999</v>
-      </c>
     </row>
     <row r="622" spans="1:9">
       <c r="A622">
@@ -18374,9 +18365,6 @@
       </c>
       <c r="H622">
         <v>192</v>
-      </c>
-      <c r="I622">
-        <v>999999</v>
       </c>
     </row>
     <row r="623" spans="1:9">

</xml_diff>